<commit_message>
Model Rack: add DCF + Precedent Transactions, extend 3-statement to 5 years
- New dcf-template.xlsx: five-year unlevered FCF discounted at WACC with a
  perpetuity-growth terminal value, EV -> equity -> implied share price.
- New precedent-transactions-template.xlsx: acquisition multiples on a deal set,
  median applied to a target on a control basis (implies a premium to trading comps).
- three-statement-template.xlsx now projects five forecast years (FY1-FY5); the
  balance sheet still ties to zero every period (verified numerically).
- Model Rack card now lists all five templates.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/models/three-statement-template.xlsx
+++ b/public/models/three-statement-template.xlsx
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -510,6 +510,8 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -522,7 +524,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>A simplified integrated model: income statement, cash flow, and a balance sheet that ties out every year.</t>
+          <t>A simplified integrated model: income statement, cash flow, and a balance sheet that ties out every year (five-year forecast).</t>
         </is>
       </c>
     </row>
@@ -557,6 +559,16 @@
       <c r="F5" s="5" t="inlineStr">
         <is>
           <t>FY3</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>FY4</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>FY5</t>
         </is>
       </c>
     </row>
@@ -571,6 +583,8 @@
       <c r="D6" s="6" t="n"/>
       <c r="E6" s="6" t="n"/>
       <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -673,6 +687,8 @@
       <c r="D16" s="6" t="n"/>
       <c r="E16" s="6" t="n"/>
       <c r="F16" s="6" t="n"/>
+      <c r="G16" s="6" t="n"/>
+      <c r="H16" s="6" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
@@ -695,6 +711,14 @@
         <f>E17*(1+$C$7)</f>
         <v/>
       </c>
+      <c r="G17" s="11">
+        <f>F17*(1+$C$7)</f>
+        <v/>
+      </c>
+      <c r="H17" s="11">
+        <f>G17*(1+$C$7)</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -718,6 +742,14 @@
         <f>-F17*$C$8</f>
         <v/>
       </c>
+      <c r="G18" s="11">
+        <f>-G17*$C$8</f>
+        <v/>
+      </c>
+      <c r="H18" s="11">
+        <f>-H17*$C$8</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -741,6 +773,14 @@
         <f>F17+F18</f>
         <v/>
       </c>
+      <c r="G19" s="12">
+        <f>G17+G18</f>
+        <v/>
+      </c>
+      <c r="H19" s="12">
+        <f>H17+H18</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -764,6 +804,14 @@
         <f>-F17*$C$9</f>
         <v/>
       </c>
+      <c r="G20" s="11">
+        <f>-G17*$C$9</f>
+        <v/>
+      </c>
+      <c r="H20" s="11">
+        <f>-H17*$C$9</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
@@ -787,6 +835,14 @@
         <f>F19+F20</f>
         <v/>
       </c>
+      <c r="G21" s="13">
+        <f>G19+G20</f>
+        <v/>
+      </c>
+      <c r="H21" s="13">
+        <f>H19+H20</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -810,6 +866,14 @@
         <f>-F17*$C$10</f>
         <v/>
       </c>
+      <c r="G22" s="11">
+        <f>-G17*$C$10</f>
+        <v/>
+      </c>
+      <c r="H22" s="11">
+        <f>-H17*$C$10</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
@@ -833,6 +897,14 @@
         <f>F21+F22</f>
         <v/>
       </c>
+      <c r="G23" s="12">
+        <f>G21+G22</f>
+        <v/>
+      </c>
+      <c r="H23" s="12">
+        <f>H21+H22</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -856,6 +928,14 @@
         <f>-F34*$C$13</f>
         <v/>
       </c>
+      <c r="G24" s="11">
+        <f>-G34*$C$13</f>
+        <v/>
+      </c>
+      <c r="H24" s="11">
+        <f>-H34*$C$13</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
@@ -879,6 +959,14 @@
         <f>F23+F24</f>
         <v/>
       </c>
+      <c r="G25" s="12">
+        <f>G23+G24</f>
+        <v/>
+      </c>
+      <c r="H25" s="12">
+        <f>H23+H24</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -902,6 +990,14 @@
         <f>-F25*$C$14</f>
         <v/>
       </c>
+      <c r="G26" s="11">
+        <f>-G25*$C$14</f>
+        <v/>
+      </c>
+      <c r="H26" s="11">
+        <f>-H25*$C$14</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
@@ -923,6 +1019,14 @@
       </c>
       <c r="F27" s="13">
         <f>F25+F26</f>
+        <v/>
+      </c>
+      <c r="G27" s="13">
+        <f>G25+G26</f>
+        <v/>
+      </c>
+      <c r="H27" s="13">
+        <f>H25+H26</f>
         <v/>
       </c>
     </row>
@@ -937,6 +1041,8 @@
       <c r="D29" s="6" t="n"/>
       <c r="E29" s="6" t="n"/>
       <c r="F29" s="6" t="n"/>
+      <c r="G29" s="6" t="n"/>
+      <c r="H29" s="6" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -959,6 +1065,14 @@
         <f>F53</f>
         <v/>
       </c>
+      <c r="G30" s="11">
+        <f>G53</f>
+        <v/>
+      </c>
+      <c r="H30" s="11">
+        <f>H53</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -982,6 +1096,14 @@
         <f>F17*$C$12</f>
         <v/>
       </c>
+      <c r="G31" s="11">
+        <f>G17*$C$12</f>
+        <v/>
+      </c>
+      <c r="H31" s="11">
+        <f>H17*$C$12</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -1004,6 +1126,14 @@
         <f>E32+F17*$C$11+F22</f>
         <v/>
       </c>
+      <c r="G32" s="11">
+        <f>F32+G17*$C$11+G22</f>
+        <v/>
+      </c>
+      <c r="H32" s="11">
+        <f>G32+H17*$C$11+H22</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
@@ -1027,6 +1157,14 @@
         <f>F30+F31+F32</f>
         <v/>
       </c>
+      <c r="G33" s="13">
+        <f>G30+G31+G32</f>
+        <v/>
+      </c>
+      <c r="H33" s="13">
+        <f>H30+H31+H32</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -1049,6 +1187,14 @@
         <f>E34</f>
         <v/>
       </c>
+      <c r="G34" s="11">
+        <f>F34</f>
+        <v/>
+      </c>
+      <c r="H34" s="11">
+        <f>G34</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="9" t="inlineStr">
@@ -1072,6 +1218,14 @@
         <f>F34</f>
         <v/>
       </c>
+      <c r="G35" s="12">
+        <f>G34</f>
+        <v/>
+      </c>
+      <c r="H35" s="12">
+        <f>H34</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -1094,6 +1248,14 @@
         <f>E36</f>
         <v/>
       </c>
+      <c r="G36" s="11">
+        <f>F36</f>
+        <v/>
+      </c>
+      <c r="H36" s="11">
+        <f>G36</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -1117,6 +1279,14 @@
         <f>E37+F27+F49</f>
         <v/>
       </c>
+      <c r="G37" s="11">
+        <f>F37+G27+G49</f>
+        <v/>
+      </c>
+      <c r="H37" s="11">
+        <f>G37+H27+H49</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
@@ -1140,6 +1310,14 @@
         <f>F36+F37</f>
         <v/>
       </c>
+      <c r="G38" s="12">
+        <f>G36+G37</f>
+        <v/>
+      </c>
+      <c r="H38" s="12">
+        <f>H36+H37</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="9" t="inlineStr">
@@ -1163,6 +1341,14 @@
         <f>F35+F38</f>
         <v/>
       </c>
+      <c r="G39" s="13">
+        <f>G35+G38</f>
+        <v/>
+      </c>
+      <c r="H39" s="13">
+        <f>H35+H38</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -1184,6 +1370,14 @@
       </c>
       <c r="F40" s="14">
         <f>F33-F39</f>
+        <v/>
+      </c>
+      <c r="G40" s="14">
+        <f>G33-G39</f>
+        <v/>
+      </c>
+      <c r="H40" s="14">
+        <f>H33-H39</f>
         <v/>
       </c>
     </row>
@@ -1198,6 +1392,8 @@
       <c r="D42" s="6" t="n"/>
       <c r="E42" s="6" t="n"/>
       <c r="F42" s="6" t="n"/>
+      <c r="G42" s="6" t="n"/>
+      <c r="H42" s="6" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -1222,6 +1418,14 @@
         <f>F27</f>
         <v/>
       </c>
+      <c r="G43" s="11">
+        <f>G27</f>
+        <v/>
+      </c>
+      <c r="H43" s="11">
+        <f>H27</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -1246,6 +1450,14 @@
         <f>-F22</f>
         <v/>
       </c>
+      <c r="G44" s="11">
+        <f>-G22</f>
+        <v/>
+      </c>
+      <c r="H44" s="11">
+        <f>-H22</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -1270,6 +1482,14 @@
         <f>-(F31-E31)</f>
         <v/>
       </c>
+      <c r="G45" s="11">
+        <f>-(G31-F31)</f>
+        <v/>
+      </c>
+      <c r="H45" s="11">
+        <f>-(H31-G31)</f>
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="9" t="inlineStr">
@@ -1294,6 +1514,14 @@
         <f>F43+F44+F45</f>
         <v/>
       </c>
+      <c r="G46" s="13">
+        <f>G43+G44+G45</f>
+        <v/>
+      </c>
+      <c r="H46" s="13">
+        <f>H43+H44+H45</f>
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -1318,6 +1546,14 @@
         <f>-F17*$C$11</f>
         <v/>
       </c>
+      <c r="G47" s="11">
+        <f>-G17*$C$11</f>
+        <v/>
+      </c>
+      <c r="H47" s="11">
+        <f>-H17*$C$11</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="9" t="inlineStr">
@@ -1342,6 +1578,14 @@
         <f>F47</f>
         <v/>
       </c>
+      <c r="G48" s="12">
+        <f>G47</f>
+        <v/>
+      </c>
+      <c r="H48" s="12">
+        <f>H47</f>
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -1366,6 +1610,14 @@
         <f>-F27*$C$15</f>
         <v/>
       </c>
+      <c r="G49" s="11">
+        <f>-G27*$C$15</f>
+        <v/>
+      </c>
+      <c r="H49" s="11">
+        <f>-H27*$C$15</f>
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="9" t="inlineStr">
@@ -1390,6 +1642,14 @@
         <f>F49</f>
         <v/>
       </c>
+      <c r="G50" s="12">
+        <f>G49</f>
+        <v/>
+      </c>
+      <c r="H50" s="12">
+        <f>H49</f>
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="9" t="inlineStr">
@@ -1414,6 +1674,14 @@
         <f>F46+F48+F50</f>
         <v/>
       </c>
+      <c r="G51" s="13">
+        <f>G46+G48+G50</f>
+        <v/>
+      </c>
+      <c r="H51" s="13">
+        <f>H46+H48+H50</f>
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -1438,6 +1706,14 @@
         <f>E30</f>
         <v/>
       </c>
+      <c r="G52" s="11">
+        <f>F30</f>
+        <v/>
+      </c>
+      <c r="H52" s="11">
+        <f>G30</f>
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="9" t="inlineStr">
@@ -1460,6 +1736,14 @@
       </c>
       <c r="F53" s="12">
         <f>F52+F51</f>
+        <v/>
+      </c>
+      <c r="G53" s="12">
+        <f>G52+G51</f>
+        <v/>
+      </c>
+      <c r="H53" s="12">
+        <f>H52+H51</f>
         <v/>
       </c>
     </row>

</xml_diff>